<commit_message>
Grilles finales : DEX 3 modes, réseaux sociaux et packs Visuo, simulateur avec recherche et impression couleur / N&B
- Tarifs, page DEX et FAQ : Mode 3 (fiche de synthèse + PowerPoint)
- Visuo : Facebook, Instagram, WhatsApp Business ; packs avec réseaux ; Pack Vitrine ; retraits demandés
- Paiement : recherche dans toutes les prestations, plusieurs lignes, pages couleur et noir et blanc
- Inscription : commissions des 3 branches, message sans réafficher le code d'accès
- generer_catalogues.py : une seule source de prix pour Excel, site et script

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TU7cV84L6MBanZjeXvtZ2A
</commit_message>
<xml_diff>
--- a/outils-factures/DWTS_Devis_Factures.xlsx
+++ b/outils-factures/DWTS_Devis_Factures.xlsx
@@ -16,12 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facture Logia" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="Articles">Grille!$D$5:$D$82</definedName>
-    <definedName name="Prix">Grille!$E$5:$E$82</definedName>
-    <definedName name="Types">Grille!$F$5:$F$82</definedName>
-    <definedName name="Liste_DEX">Grille!$D$5:$D$26</definedName>
-    <definedName name="Liste_Visuo">Grille!$D$28:$D$63</definedName>
-    <definedName name="Liste_Logia">Grille!$D$65:$D$82</definedName>
+    <definedName name="Articles">Grille!$D$5:$D$91</definedName>
+    <definedName name="Prix">Grille!$E$5:$E$91</definedName>
+    <definedName name="Types">Grille!$F$5:$F$91</definedName>
+    <definedName name="Liste_DEX">Grille!$D$5:$D$36</definedName>
+    <definedName name="Liste_Visuo">Grille!$D$38:$D$72</definedName>
+    <definedName name="Liste_Logia">Grille!$D$74:$D$91</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Devis Visuo'!$A$1:$E$41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Devis Logia'!$A$1:$E$40</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Facture DEX'!$A$1:$D$26</definedName>
@@ -1103,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1228,21 +1228,21 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 2 (5 à 9 pages ou images)</t>
+          <t>Exposé palier 1 (4 pages ou moins)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 1</t>
+          <t>Exposé palier 1 (4 pages ou moins) · Mode 3</t>
         </is>
       </c>
       <c r="E7" s="8" t="n">
-        <v>4000</v>
+        <v>7000</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
@@ -1263,16 +1263,16 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 2</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 1</t>
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>5500</v>
+        <v>4000</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 3 (10 pages ou plus)</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images)</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 3 (10 pages ou plus) · Mode 1</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 2</t>
         </is>
       </c>
       <c r="E9" s="8" t="n">
@@ -1318,21 +1318,21 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 3 (10 pages ou plus)</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images)</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 3 (10 pages ou plus) · Mode 2</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 3</t>
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>7000</v>
+        <v>8500</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
+          <t>Exposé palier 3 (10 pages ou plus)</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 1</t>
+          <t>Exposé palier 3 (10 pages ou plus) · Mode 1</t>
         </is>
       </c>
       <c r="E11" s="8" t="n">
-        <v>7000</v>
+        <v>5500</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
+          <t>Exposé palier 3 (10 pages ou plus)</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -1388,11 +1388,11 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 2</t>
+          <t>Exposé palier 3 (10 pages ou plus) · Mode 2</t>
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>8500</v>
+        <v>7000</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -1408,21 +1408,21 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
+          <t>Exposé palier 3 (10 pages ou plus)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 1</t>
+          <t>Exposé palier 3 (10 pages ou plus) · Mode 3</t>
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>8500</v>
+        <v>10000</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
@@ -1438,21 +1438,21 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 2</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 1</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>10000</v>
+        <v>7000</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -1468,21 +1468,21 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>CV + lettre de motivation</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>CV + lettre de motivation · Mode 1</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 2</t>
         </is>
       </c>
       <c r="E15" s="8" t="n">
-        <v>1500</v>
+        <v>8500</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>CV + lettre de motivation</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>CV + lettre de motivation · Mode 2</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 3</t>
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>3000</v>
+        <v>11500</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Rapport de stage</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -1538,11 +1538,11 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Rapport de stage · Mode 1</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 1</t>
         </is>
       </c>
       <c r="E17" s="8" t="n">
-        <v>7500</v>
+        <v>8500</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Rapport de stage</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -1568,11 +1568,11 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Rapport de stage · Mode 2</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 2</t>
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>10500</v>
+        <v>10000</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -1588,21 +1588,21 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Mémoire Bac+1 à Bac+3</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Mémoire Bac+1 à Bac+3 · Mode 1</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 3</t>
         </is>
       </c>
       <c r="E19" s="8" t="n">
-        <v>10500</v>
+        <v>13000</v>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
@@ -1618,21 +1618,21 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Mémoire Bac+1 à Bac+3</t>
+          <t>CV + lettre de motivation</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Mémoire Bac+1 à Bac+3 · Mode 2</t>
+          <t>CV + lettre de motivation · Mode 1</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
-        <v>13500</v>
+        <v>1500</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Document professionnel</t>
+          <t>CV + lettre de motivation</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Document professionnel · Mode 1</t>
+          <t>CV + lettre de motivation · Mode 2</t>
         </is>
       </c>
       <c r="E21" s="8" t="n">
-        <v>10500</v>
+        <v>3000</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -1678,21 +1678,21 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Document professionnel</t>
+          <t>CV + lettre de motivation</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Document professionnel · Mode 2</t>
+          <t>CV + lettre de motivation · Mode 3</t>
         </is>
       </c>
       <c r="E22" s="8" t="n">
-        <v>15500</v>
+        <v>4500</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Master et thèse</t>
+          <t>Rapport de stage</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -1718,11 +1718,11 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Master et thèse · Mode 1</t>
+          <t>Rapport de stage · Mode 1</t>
         </is>
       </c>
       <c r="E23" s="8" t="n">
-        <v>15500</v>
+        <v>7500</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Master et thèse</t>
+          <t>Rapport de stage</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1748,11 +1748,11 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Master et thèse · Mode 2</t>
+          <t>Rapport de stage · Mode 2</t>
         </is>
       </c>
       <c r="E24" s="8" t="n">
-        <v>18500</v>
+        <v>10500</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
@@ -1768,21 +1768,21 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Impression page couleur</t>
+          <t>Rapport de stage</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Par page</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Impression page couleur</t>
+          <t>Rapport de stage · Mode 3</t>
         </is>
       </c>
       <c r="E25" s="8" t="n">
-        <v>500</v>
+        <v>14500</v>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
@@ -1798,23 +1798,53 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Impression page noir et blanc</t>
+          <t>Mémoire Bac+1 à Bac+3</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Par page</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Impression page noir et blanc</t>
+          <t>Mémoire Bac+1 à Bac+3 · Mode 1</t>
         </is>
       </c>
       <c r="E26" s="8" t="n">
-        <v>200</v>
+        <v>10500</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Mémoire Bac+1 à Bac+3</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Mode 2</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Mémoire Bac+1 à Bac+3 · Mode 2</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>13500</v>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
@@ -1823,26 +1853,26 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Mémoire Bac+1 à Bac+3</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Logo · Basique</t>
+          <t>Mémoire Bac+1 à Bac+3 · Mode 3</t>
         </is>
       </c>
       <c r="E28" s="8" t="n">
-        <v>6500</v>
+        <v>18500</v>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
@@ -1853,26 +1883,26 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Document professionnel</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Logo · Standard</t>
+          <t>Document professionnel · Mode 1</t>
         </is>
       </c>
       <c r="E29" s="8" t="n">
-        <v>10000</v>
+        <v>10500</v>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
@@ -1883,26 +1913,26 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Document professionnel</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Logo · Premium</t>
+          <t>Document professionnel · Mode 2</t>
         </is>
       </c>
       <c r="E30" s="8" t="n">
-        <v>15000</v>
+        <v>15500</v>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
@@ -1913,26 +1943,26 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer</t>
+          <t>Document professionnel</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer · Basique</t>
+          <t>Document professionnel · Mode 3</t>
         </is>
       </c>
       <c r="E31" s="8" t="n">
-        <v>2500</v>
+        <v>19500</v>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
@@ -1943,26 +1973,26 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer</t>
+          <t>Master et thèse</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer · Standard</t>
+          <t>Master et thèse · Mode 1</t>
         </is>
       </c>
       <c r="E32" s="8" t="n">
-        <v>4000</v>
+        <v>15500</v>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
@@ -1973,26 +2003,26 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer</t>
+          <t>Master et thèse</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer · Premium</t>
+          <t>Master et thèse · Mode 2</t>
         </is>
       </c>
       <c r="E33" s="8" t="n">
-        <v>6000</v>
+        <v>18500</v>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
@@ -2003,26 +2033,26 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation</t>
+          <t>Master et thèse</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation · Basique</t>
+          <t>Master et thèse · Mode 3</t>
         </is>
       </c>
       <c r="E34" s="8" t="n">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
@@ -2033,26 +2063,26 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation</t>
+          <t>Impression page couleur</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Par page</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation · Standard</t>
+          <t>Impression page couleur</t>
         </is>
       </c>
       <c r="E35" s="8" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
@@ -2063,58 +2093,28 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation</t>
+          <t>Impression page noir et blanc</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Par page</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation · Premium</t>
+          <t>Impression page noir et blanc</t>
         </is>
       </c>
       <c r="E36" s="8" t="n">
-        <v>5000</v>
+        <v>200</v>
       </c>
       <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Unique</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>Visuo</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Carte de visite</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>Basique</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Carte de visite · Basique</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
@@ -2128,21 +2128,21 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Carte de visite</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Carte de visite · Standard</t>
+          <t>Logo · Basique</t>
         </is>
       </c>
       <c r="E38" s="8" t="n">
-        <v>3000</v>
+        <v>6500</v>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
@@ -2158,21 +2158,21 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Carte de visite</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Carte de visite · Premium</t>
+          <t>Logo · Standard</t>
         </is>
       </c>
       <c r="E39" s="8" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
@@ -2188,21 +2188,21 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis · Basique</t>
+          <t>Logo · Premium</t>
         </is>
       </c>
       <c r="E40" s="8" t="n">
-        <v>2500</v>
+        <v>15000</v>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
@@ -2218,21 +2218,21 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis</t>
+          <t>Affiche ou flyer</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis · Standard</t>
+          <t>Affiche ou flyer · Basique</t>
         </is>
       </c>
       <c r="E41" s="8" t="n">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis</t>
+          <t>Affiche ou flyer</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis · Premium</t>
+          <t>Affiche ou flyer · Standard</t>
         </is>
       </c>
       <c r="E42" s="8" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
@@ -2278,21 +2278,21 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s</t>
+          <t>Affiche ou flyer</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s · Basique</t>
+          <t>Affiche ou flyer · Premium</t>
         </is>
       </c>
       <c r="E43" s="8" t="n">
-        <v>7500</v>
+        <v>6000</v>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
@@ -2308,21 +2308,21 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s</t>
+          <t>Carte d'invitation</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s · Standard</t>
+          <t>Carte d'invitation · Basique</t>
         </is>
       </c>
       <c r="E44" s="8" t="n">
-        <v>9500</v>
+        <v>2000</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
@@ -2338,21 +2338,21 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s</t>
+          <t>Carte d'invitation</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s · Premium</t>
+          <t>Carte d'invitation · Standard</t>
         </is>
       </c>
       <c r="E45" s="8" t="n">
-        <v>15000</v>
+        <v>3000</v>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
@@ -2368,21 +2368,21 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine</t>
+          <t>Carte d'invitation</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine · Basique</t>
+          <t>Carte d'invitation · Premium</t>
         </is>
       </c>
       <c r="E46" s="8" t="n">
-        <v>12500</v>
+        <v>5000</v>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine</t>
+          <t>Carte de visite</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine · Standard</t>
+          <t>Carte de visite · Basique</t>
         </is>
       </c>
       <c r="E47" s="8" t="n">
-        <v>25000</v>
+        <v>2000</v>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
@@ -2428,21 +2428,21 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine</t>
+          <t>Carte de visite</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine · Premium</t>
+          <t>Carte de visite · Standard</t>
         </is>
       </c>
       <c r="E48" s="8" t="n">
-        <v>45000</v>
+        <v>3000</v>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
@@ -2458,25 +2458,25 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site</t>
+          <t>Carte de visite</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site · Basique</t>
+          <t>Carte de visite · Premium</t>
         </is>
       </c>
       <c r="E49" s="8" t="n">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2488,25 +2488,25 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ)</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site · Standard</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ) · Basique</t>
         </is>
       </c>
       <c r="E50" s="8" t="n">
-        <v>5000</v>
+        <v>7500</v>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2518,25 +2518,25 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ)</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site · Premium</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ) · Standard</t>
         </is>
       </c>
       <c r="E51" s="8" t="n">
-        <v>10000</v>
+        <v>9500</v>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2548,25 +2548,25 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ)</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages · Basique</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ) · Premium</t>
         </is>
       </c>
       <c r="E52" s="8" t="n">
-        <v>7000</v>
+        <v>15000</v>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2578,17 +2578,17 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages</t>
+          <t>Site vitrine</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages · Standard</t>
+          <t>Site vitrine · Basique</t>
         </is>
       </c>
       <c r="E53" s="8" t="n">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2608,25 +2608,25 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages</t>
+          <t>Site vitrine</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages · Premium</t>
+          <t>Site vitrine · Standard</t>
         </is>
       </c>
       <c r="E54" s="8" t="n">
-        <v>22000</v>
+        <v>25000</v>
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2638,25 +2638,25 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Gestion du compte WhatsApp</t>
+          <t>Site vitrine</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Toutes formules</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Gestion du compte WhatsApp</t>
+          <t>Site vitrine · Premium</t>
         </is>
       </c>
       <c r="E55" s="8" t="n">
-        <v>10000</v>
+        <v>45000</v>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2668,25 +2668,25 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Publication réseaux</t>
+          <t>Maintenance du site</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>À l'unité</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Publication réseaux</t>
+          <t>Maintenance du site · Basique</t>
         </is>
       </c>
       <c r="E56" s="8" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
@@ -2698,21 +2698,21 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter (1 affiche, 4 publications)</t>
+          <t>Maintenance du site</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter (1 affiche, 4 publications)</t>
+          <t>Maintenance du site · Standard</t>
         </is>
       </c>
       <c r="E57" s="8" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
@@ -2728,21 +2728,21 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Pack Basique (2 affiches, 8 publications, 1 vidéo)</t>
+          <t>Maintenance du site</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Pack Basique (2 affiches, 8 publications, 1 vidéo)</t>
+          <t>Maintenance du site · Premium</t>
         </is>
       </c>
       <c r="E58" s="8" t="n">
-        <v>18000</v>
+        <v>10000</v>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
@@ -2758,21 +2758,21 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Pack Standard (4 affiches, 12 publications, 2 vidéos, maintenance)</t>
+          <t>Gestion de la page Facebook</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Pack Standard (4 affiches, 12 publications, 2 vidéos, maintenance)</t>
+          <t>Gestion de la page Facebook · Basique</t>
         </is>
       </c>
       <c r="E59" s="8" t="n">
-        <v>50000</v>
+        <v>7000</v>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
@@ -2788,21 +2788,21 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Pack Premium (6 affiches, 20 publications, 4 vidéos, maintenance)</t>
+          <t>Gestion de la page Facebook</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Pack Premium (6 affiches, 20 publications, 4 vidéos, maintenance)</t>
+          <t>Gestion de la page Facebook · Standard</t>
         </is>
       </c>
       <c r="E60" s="8" t="n">
-        <v>115000</v>
+        <v>12500</v>
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
@@ -2818,25 +2818,25 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack</t>
+          <t>Gestion de la page Facebook</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack · Basique</t>
+          <t>Gestion de la page Facebook · Premium</t>
         </is>
       </c>
       <c r="E61" s="8" t="n">
-        <v>15000</v>
+        <v>22000</v>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
@@ -2848,25 +2848,25 @@
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack</t>
+          <t>Gestion du compte Instagram</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack · Standard</t>
+          <t>Gestion du compte Instagram · Basique</t>
         </is>
       </c>
       <c r="E62" s="8" t="n">
-        <v>28000</v>
+        <v>8000</v>
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
@@ -2878,37 +2878,67 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack</t>
+          <t>Gestion du compte Instagram</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Gestion du compte Instagram · Standard</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>Visuo</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Gestion du compte Instagram</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>Site + facture avec un pack · Premium</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="n">
-        <v>50000</v>
-      </c>
-      <c r="F63" s="7" t="inlineStr">
-        <is>
-          <t>Unique</t>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Gestion du compte Instagram · Premium</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="n">
+        <v>24500</v>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Automatisation</t>
+          <t>Gestion du compte WhatsApp Business</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
@@ -2918,27 +2948,27 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>Automatisation · Basique</t>
+          <t>Gestion du compte WhatsApp Business · Basique</t>
         </is>
       </c>
       <c r="E65" s="8" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Automatisation</t>
+          <t>Gestion du compte WhatsApp Business</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
@@ -2948,27 +2978,27 @@
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Automatisation · Standard</t>
+          <t>Gestion du compte WhatsApp Business · Standard</t>
         </is>
       </c>
       <c r="E66" s="8" t="n">
-        <v>15000</v>
+        <v>11500</v>
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Automatisation</t>
+          <t>Gestion du compte WhatsApp Business</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
@@ -2978,193 +3008,163 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Automatisation · Premium</t>
+          <t>Gestion du compte WhatsApp Business · Premium</t>
         </is>
       </c>
       <c r="E67" s="8" t="n">
-        <v>30000</v>
+        <v>20500</v>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp</t>
+          <t>Pack Starter (Facebook ; 1 affiche, 4 publications)</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp · Basique</t>
+          <t>Pack Starter (Facebook ; 1 affiche, 4 publications)</t>
         </is>
       </c>
       <c r="E68" s="8" t="n">
-        <v>15000</v>
+        <v>6000</v>
       </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp</t>
+          <t>Pack Basique (Facebook + WhatsApp Business ; 2 affiches, 8 publications, 1 vidéo)</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp · Standard</t>
+          <t>Pack Basique (Facebook + WhatsApp Business ; 2 affiches, 8 publications, 1 vidéo)</t>
         </is>
       </c>
       <c r="E69" s="8" t="n">
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp</t>
+          <t>Pack Standard (Facebook + Instagram + WhatsApp Business ; 4 affiches, 12 publications, 2 vidéos, maintenance du site)</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp · Premium</t>
+          <t>Pack Standard (Facebook + Instagram + WhatsApp Business ; 4 affiches, 12 publications, 2 vidéos, maintenance du site)</t>
         </is>
       </c>
       <c r="E70" s="8" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Logiciel de gestion</t>
+          <t>Pack Premium (Facebook + Instagram + WhatsApp Business ; 6 affiches, 20 publications, 4 vidéos, maintenance du site)</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Logiciel de gestion · Basique</t>
+          <t>Pack Premium (Facebook + Instagram + WhatsApp Business ; 6 affiches, 20 publications, 4 vidéos, maintenance du site)</t>
         </is>
       </c>
       <c r="E71" s="8" t="n">
-        <v>45000</v>
+        <v>115000</v>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Logiciel de gestion</t>
+          <t>Pack Vitrine (site vitrine Basique + 1er mois du Pack Basique, puis 18 000 / mois)</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>Logiciel de gestion · Standard</t>
+          <t>Pack Vitrine (site vitrine Basique + 1er mois du Pack Basique, puis 18 000 / mois)</t>
         </is>
       </c>
       <c r="E72" s="8" t="n">
-        <v>90000</v>
+        <v>28000</v>
       </c>
       <c r="F72" s="7" t="inlineStr">
-        <is>
-          <t>Unique</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="7" t="inlineStr">
-        <is>
-          <t>Logia</t>
-        </is>
-      </c>
-      <c r="B73" s="7" t="inlineStr">
-        <is>
-          <t>Logiciel de gestion</t>
-        </is>
-      </c>
-      <c r="C73" s="7" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t>Logiciel de gestion · Premium</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F73" s="7" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
@@ -3178,7 +3178,7 @@
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>Suivi</t>
+          <t>Automatisation</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
@@ -3188,15 +3188,15 @@
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>Suivi · Basique</t>
+          <t>Automatisation · Basique</t>
         </is>
       </c>
       <c r="E74" s="8" t="n">
-        <v>5000</v>
+        <v>7500</v>
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Suivi</t>
+          <t>Automatisation</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
@@ -3218,15 +3218,15 @@
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>Suivi · Standard</t>
+          <t>Automatisation · Standard</t>
         </is>
       </c>
       <c r="E75" s="8" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>Suivi</t>
+          <t>Automatisation</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
@@ -3248,15 +3248,15 @@
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>Suivi · Premium</t>
+          <t>Automatisation · Premium</t>
         </is>
       </c>
       <c r="E76" s="8" t="n">
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3268,21 +3268,21 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter : mise en service</t>
+          <t>Bot WhatsApp</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter : mise en service</t>
+          <t>Bot WhatsApp · Basique</t>
         </is>
       </c>
       <c r="E77" s="8" t="n">
-        <v>7500</v>
+        <v>15000</v>
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
@@ -3298,25 +3298,25 @@
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter : suivi</t>
+          <t>Bot WhatsApp</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter : suivi</t>
+          <t>Bot WhatsApp · Standard</t>
         </is>
       </c>
       <c r="E78" s="8" t="n">
-        <v>5000</v>
+        <v>30000</v>
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3328,21 +3328,21 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Pack Business : mise en service</t>
+          <t>Bot WhatsApp</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>Pack Business : mise en service</t>
+          <t>Bot WhatsApp · Premium</t>
         </is>
       </c>
       <c r="E79" s="8" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
@@ -3358,25 +3358,25 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>Pack Business : suivi</t>
+          <t>Logiciel de gestion</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>Pack Business : suivi</t>
+          <t>Logiciel de gestion · Basique</t>
         </is>
       </c>
       <c r="E80" s="8" t="n">
-        <v>10000</v>
+        <v>45000</v>
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3388,21 +3388,21 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Pack Entreprise : mise en service</t>
+          <t>Logiciel de gestion</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>Pack Entreprise : mise en service</t>
+          <t>Logiciel de gestion · Standard</t>
         </is>
       </c>
       <c r="E81" s="8" t="n">
-        <v>110000</v>
+        <v>90000</v>
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
@@ -3418,23 +3418,293 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
+          <t>Logiciel de gestion</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Logiciel de gestion · Premium</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="n">
+        <v>180000</v>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Suivi</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Basique</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Suivi · Basique</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Suivi</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>Suivi · Standard</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Suivi</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>Suivi · Premium</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Pack Starter : mise en service</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>Pack Starter : mise en service</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Pack Starter : suivi</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>Pack Starter : suivi</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Pack Business : mise en service</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr">
+        <is>
+          <t>Pack Business : mise en service</t>
+        </is>
+      </c>
+      <c r="E88" s="8" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F88" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Pack Business : suivi</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>Pack Business : suivi</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>Pack Entreprise : mise en service</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>Pack Entreprise : mise en service</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="n">
+        <v>110000</v>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
           <t>Pack Entreprise : suivi</t>
         </is>
       </c>
-      <c r="C82" s="7" t="inlineStr">
+      <c r="C91" s="7" t="inlineStr">
         <is>
           <t>Pack</t>
         </is>
       </c>
-      <c r="D82" s="7" t="inlineStr">
+      <c r="D91" s="7" t="inlineStr">
         <is>
           <t>Pack Entreprise : suivi</t>
         </is>
       </c>
-      <c r="E82" s="8" t="n">
+      <c r="E91" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="F82" s="7" t="inlineStr">
+      <c r="F91" s="7" t="inlineStr">
         <is>
           <t>Mensuel</t>
         </is>

</xml_diff>

<commit_message>
Grilles finales : DEX 3 modes, réseaux sociaux et packs Visuo, simulateur avec recherche et impression couleur / N&B (#18)
- Tarifs, page DEX et FAQ : Mode 3 (fiche de synthèse + PowerPoint)
- Visuo : Facebook, Instagram, WhatsApp Business ; packs avec réseaux ; Pack Vitrine ; retraits demandés
- Paiement : recherche dans toutes les prestations, plusieurs lignes, pages couleur et noir et blanc
- Inscription : commissions des 3 branches, message sans réafficher le code d'accès
- generer_catalogues.py : une seule source de prix pour Excel, site et script


Claude-Session: https://claude.ai/code/session_01TU7cV84L6MBanZjeXvtZ2A

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outils-factures/DWTS_Devis_Factures.xlsx
+++ b/outils-factures/DWTS_Devis_Factures.xlsx
@@ -16,12 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facture Logia" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="Articles">Grille!$D$5:$D$82</definedName>
-    <definedName name="Prix">Grille!$E$5:$E$82</definedName>
-    <definedName name="Types">Grille!$F$5:$F$82</definedName>
-    <definedName name="Liste_DEX">Grille!$D$5:$D$26</definedName>
-    <definedName name="Liste_Visuo">Grille!$D$28:$D$63</definedName>
-    <definedName name="Liste_Logia">Grille!$D$65:$D$82</definedName>
+    <definedName name="Articles">Grille!$D$5:$D$91</definedName>
+    <definedName name="Prix">Grille!$E$5:$E$91</definedName>
+    <definedName name="Types">Grille!$F$5:$F$91</definedName>
+    <definedName name="Liste_DEX">Grille!$D$5:$D$36</definedName>
+    <definedName name="Liste_Visuo">Grille!$D$38:$D$72</definedName>
+    <definedName name="Liste_Logia">Grille!$D$74:$D$91</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Devis Visuo'!$A$1:$E$41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Devis Logia'!$A$1:$E$40</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Facture DEX'!$A$1:$D$26</definedName>
@@ -1103,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1228,21 +1228,21 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 2 (5 à 9 pages ou images)</t>
+          <t>Exposé palier 1 (4 pages ou moins)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 1</t>
+          <t>Exposé palier 1 (4 pages ou moins) · Mode 3</t>
         </is>
       </c>
       <c r="E7" s="8" t="n">
-        <v>4000</v>
+        <v>7000</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
@@ -1263,16 +1263,16 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 2</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 1</t>
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>5500</v>
+        <v>4000</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
@@ -1288,17 +1288,17 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 3 (10 pages ou plus)</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images)</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 3 (10 pages ou plus) · Mode 1</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 2</t>
         </is>
       </c>
       <c r="E9" s="8" t="n">
@@ -1318,21 +1318,21 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 3 (10 pages ou plus)</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images)</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 3 (10 pages ou plus) · Mode 2</t>
+          <t>Exposé palier 2 (5 à 9 pages ou images) · Mode 3</t>
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>7000</v>
+        <v>8500</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
+          <t>Exposé palier 3 (10 pages ou plus)</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 1</t>
+          <t>Exposé palier 3 (10 pages ou plus) · Mode 1</t>
         </is>
       </c>
       <c r="E11" s="8" t="n">
-        <v>7000</v>
+        <v>5500</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
+          <t>Exposé palier 3 (10 pages ou plus)</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -1388,11 +1388,11 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 2</t>
+          <t>Exposé palier 3 (10 pages ou plus) · Mode 2</t>
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>8500</v>
+        <v>7000</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -1408,21 +1408,21 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
+          <t>Exposé palier 3 (10 pages ou plus)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 1</t>
+          <t>Exposé palier 3 (10 pages ou plus) · Mode 3</t>
         </is>
       </c>
       <c r="E13" s="8" t="n">
-        <v>8500</v>
+        <v>10000</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
@@ -1438,21 +1438,21 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 2</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 1</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>10000</v>
+        <v>7000</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -1468,21 +1468,21 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>CV + lettre de motivation</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>CV + lettre de motivation · Mode 1</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 2</t>
         </is>
       </c>
       <c r="E15" s="8" t="n">
-        <v>1500</v>
+        <v>8500</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>CV + lettre de motivation</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages)</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>CV + lettre de motivation · Mode 2</t>
+          <t>Exposé palier 4 (tableaux, 10 à 14 pages) · Mode 3</t>
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>3000</v>
+        <v>11500</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Rapport de stage</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -1538,11 +1538,11 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Rapport de stage · Mode 1</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 1</t>
         </is>
       </c>
       <c r="E17" s="8" t="n">
-        <v>7500</v>
+        <v>8500</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Rapport de stage</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -1568,11 +1568,11 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Rapport de stage · Mode 2</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 2</t>
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>10500</v>
+        <v>10000</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -1588,21 +1588,21 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Mémoire Bac+1 à Bac+3</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus)</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Mémoire Bac+1 à Bac+3 · Mode 1</t>
+          <t>Exposé palier 5 (tableaux, 15 pages ou plus) · Mode 3</t>
         </is>
       </c>
       <c r="E19" s="8" t="n">
-        <v>10500</v>
+        <v>13000</v>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
@@ -1618,21 +1618,21 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Mémoire Bac+1 à Bac+3</t>
+          <t>CV + lettre de motivation</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Mémoire Bac+1 à Bac+3 · Mode 2</t>
+          <t>CV + lettre de motivation · Mode 1</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
-        <v>13500</v>
+        <v>1500</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Document professionnel</t>
+          <t>CV + lettre de motivation</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Mode 1</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Document professionnel · Mode 1</t>
+          <t>CV + lettre de motivation · Mode 2</t>
         </is>
       </c>
       <c r="E21" s="8" t="n">
-        <v>10500</v>
+        <v>3000</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -1678,21 +1678,21 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Document professionnel</t>
+          <t>CV + lettre de motivation</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Mode 2</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Document professionnel · Mode 2</t>
+          <t>CV + lettre de motivation · Mode 3</t>
         </is>
       </c>
       <c r="E22" s="8" t="n">
-        <v>15500</v>
+        <v>4500</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Master et thèse</t>
+          <t>Rapport de stage</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -1718,11 +1718,11 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Master et thèse · Mode 1</t>
+          <t>Rapport de stage · Mode 1</t>
         </is>
       </c>
       <c r="E23" s="8" t="n">
-        <v>15500</v>
+        <v>7500</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Master et thèse</t>
+          <t>Rapport de stage</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1748,11 +1748,11 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Master et thèse · Mode 2</t>
+          <t>Rapport de stage · Mode 2</t>
         </is>
       </c>
       <c r="E24" s="8" t="n">
-        <v>18500</v>
+        <v>10500</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
@@ -1768,21 +1768,21 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Impression page couleur</t>
+          <t>Rapport de stage</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Par page</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Impression page couleur</t>
+          <t>Rapport de stage · Mode 3</t>
         </is>
       </c>
       <c r="E25" s="8" t="n">
-        <v>500</v>
+        <v>14500</v>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
@@ -1798,23 +1798,53 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Impression page noir et blanc</t>
+          <t>Mémoire Bac+1 à Bac+3</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Par page</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Impression page noir et blanc</t>
+          <t>Mémoire Bac+1 à Bac+3 · Mode 1</t>
         </is>
       </c>
       <c r="E26" s="8" t="n">
-        <v>200</v>
+        <v>10500</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>DEX</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Mémoire Bac+1 à Bac+3</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Mode 2</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Mémoire Bac+1 à Bac+3 · Mode 2</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>13500</v>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
@@ -1823,26 +1853,26 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Mémoire Bac+1 à Bac+3</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Logo · Basique</t>
+          <t>Mémoire Bac+1 à Bac+3 · Mode 3</t>
         </is>
       </c>
       <c r="E28" s="8" t="n">
-        <v>6500</v>
+        <v>18500</v>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
@@ -1853,26 +1883,26 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Document professionnel</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Logo · Standard</t>
+          <t>Document professionnel · Mode 1</t>
         </is>
       </c>
       <c r="E29" s="8" t="n">
-        <v>10000</v>
+        <v>10500</v>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
@@ -1883,26 +1913,26 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Document professionnel</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Logo · Premium</t>
+          <t>Document professionnel · Mode 2</t>
         </is>
       </c>
       <c r="E30" s="8" t="n">
-        <v>15000</v>
+        <v>15500</v>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
@@ -1913,26 +1943,26 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer</t>
+          <t>Document professionnel</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer · Basique</t>
+          <t>Document professionnel · Mode 3</t>
         </is>
       </c>
       <c r="E31" s="8" t="n">
-        <v>2500</v>
+        <v>19500</v>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
@@ -1943,26 +1973,26 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer</t>
+          <t>Master et thèse</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Mode 1</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer · Standard</t>
+          <t>Master et thèse · Mode 1</t>
         </is>
       </c>
       <c r="E32" s="8" t="n">
-        <v>4000</v>
+        <v>15500</v>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
@@ -1973,26 +2003,26 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer</t>
+          <t>Master et thèse</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Mode 2</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Affiche ou flyer · Premium</t>
+          <t>Master et thèse · Mode 2</t>
         </is>
       </c>
       <c r="E33" s="8" t="n">
-        <v>6000</v>
+        <v>18500</v>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
@@ -2003,26 +2033,26 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation</t>
+          <t>Master et thèse</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Mode 3</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation · Basique</t>
+          <t>Master et thèse · Mode 3</t>
         </is>
       </c>
       <c r="E34" s="8" t="n">
-        <v>2000</v>
+        <v>25000</v>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
@@ -2033,26 +2063,26 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation</t>
+          <t>Impression page couleur</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Par page</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation · Standard</t>
+          <t>Impression page couleur</t>
         </is>
       </c>
       <c r="E35" s="8" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
@@ -2063,58 +2093,28 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Visuo</t>
+          <t>DEX</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation</t>
+          <t>Impression page noir et blanc</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Par page</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Carte d'invitation · Premium</t>
+          <t>Impression page noir et blanc</t>
         </is>
       </c>
       <c r="E36" s="8" t="n">
-        <v>5000</v>
+        <v>200</v>
       </c>
       <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Unique</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>Visuo</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Carte de visite</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>Basique</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Carte de visite · Basique</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
@@ -2128,21 +2128,21 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Carte de visite</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Carte de visite · Standard</t>
+          <t>Logo · Basique</t>
         </is>
       </c>
       <c r="E38" s="8" t="n">
-        <v>3000</v>
+        <v>6500</v>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
@@ -2158,21 +2158,21 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Carte de visite</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Carte de visite · Premium</t>
+          <t>Logo · Standard</t>
         </is>
       </c>
       <c r="E39" s="8" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
@@ -2188,21 +2188,21 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis · Basique</t>
+          <t>Logo · Premium</t>
         </is>
       </c>
       <c r="E40" s="8" t="n">
-        <v>2500</v>
+        <v>15000</v>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
@@ -2218,21 +2218,21 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis</t>
+          <t>Affiche ou flyer</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis · Standard</t>
+          <t>Affiche ou flyer · Basique</t>
         </is>
       </c>
       <c r="E41" s="8" t="n">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis</t>
+          <t>Affiche ou flyer</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Modèle de facture ou devis · Premium</t>
+          <t>Affiche ou flyer · Standard</t>
         </is>
       </c>
       <c r="E42" s="8" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
@@ -2278,21 +2278,21 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s</t>
+          <t>Affiche ou flyer</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s · Basique</t>
+          <t>Affiche ou flyer · Premium</t>
         </is>
       </c>
       <c r="E43" s="8" t="n">
-        <v>7500</v>
+        <v>6000</v>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
@@ -2308,21 +2308,21 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s</t>
+          <t>Carte d'invitation</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s · Standard</t>
+          <t>Carte d'invitation · Basique</t>
         </is>
       </c>
       <c r="E44" s="8" t="n">
-        <v>9500</v>
+        <v>2000</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
@@ -2338,21 +2338,21 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s</t>
+          <t>Carte d'invitation</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Vidéo publicitaire 15 à 30 s · Premium</t>
+          <t>Carte d'invitation · Standard</t>
         </is>
       </c>
       <c r="E45" s="8" t="n">
-        <v>15000</v>
+        <v>3000</v>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
@@ -2368,21 +2368,21 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine</t>
+          <t>Carte d'invitation</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine · Basique</t>
+          <t>Carte d'invitation · Premium</t>
         </is>
       </c>
       <c r="E46" s="8" t="n">
-        <v>12500</v>
+        <v>5000</v>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine</t>
+          <t>Carte de visite</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine · Standard</t>
+          <t>Carte de visite · Basique</t>
         </is>
       </c>
       <c r="E47" s="8" t="n">
-        <v>25000</v>
+        <v>2000</v>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
@@ -2428,21 +2428,21 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine</t>
+          <t>Carte de visite</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Site vitrine · Premium</t>
+          <t>Carte de visite · Standard</t>
         </is>
       </c>
       <c r="E48" s="8" t="n">
-        <v>45000</v>
+        <v>3000</v>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
@@ -2458,25 +2458,25 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site</t>
+          <t>Carte de visite</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site · Basique</t>
+          <t>Carte de visite · Premium</t>
         </is>
       </c>
       <c r="E49" s="8" t="n">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2488,25 +2488,25 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ)</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site · Standard</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ) · Basique</t>
         </is>
       </c>
       <c r="E50" s="8" t="n">
-        <v>5000</v>
+        <v>7500</v>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2518,25 +2518,25 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ)</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Maintenance du site · Premium</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ) · Standard</t>
         </is>
       </c>
       <c r="E51" s="8" t="n">
-        <v>10000</v>
+        <v>9500</v>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2548,25 +2548,25 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ)</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages · Basique</t>
+          <t>Vidéo publicitaire (à partir de 15 s, prix de départ) · Premium</t>
         </is>
       </c>
       <c r="E52" s="8" t="n">
-        <v>7000</v>
+        <v>15000</v>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2578,17 +2578,17 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages</t>
+          <t>Site vitrine</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages · Standard</t>
+          <t>Site vitrine · Basique</t>
         </is>
       </c>
       <c r="E53" s="8" t="n">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2608,25 +2608,25 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages</t>
+          <t>Site vitrine</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Gestion des pages · Premium</t>
+          <t>Site vitrine · Standard</t>
         </is>
       </c>
       <c r="E54" s="8" t="n">
-        <v>22000</v>
+        <v>25000</v>
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2638,25 +2638,25 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Gestion du compte WhatsApp</t>
+          <t>Site vitrine</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Toutes formules</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Gestion du compte WhatsApp</t>
+          <t>Site vitrine · Premium</t>
         </is>
       </c>
       <c r="E55" s="8" t="n">
-        <v>10000</v>
+        <v>45000</v>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -2668,25 +2668,25 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Publication réseaux</t>
+          <t>Maintenance du site</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>À l'unité</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Publication réseaux</t>
+          <t>Maintenance du site · Basique</t>
         </is>
       </c>
       <c r="E56" s="8" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
@@ -2698,21 +2698,21 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter (1 affiche, 4 publications)</t>
+          <t>Maintenance du site</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter (1 affiche, 4 publications)</t>
+          <t>Maintenance du site · Standard</t>
         </is>
       </c>
       <c r="E57" s="8" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
@@ -2728,21 +2728,21 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Pack Basique (2 affiches, 8 publications, 1 vidéo)</t>
+          <t>Maintenance du site</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Pack Basique (2 affiches, 8 publications, 1 vidéo)</t>
+          <t>Maintenance du site · Premium</t>
         </is>
       </c>
       <c r="E58" s="8" t="n">
-        <v>18000</v>
+        <v>10000</v>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
@@ -2758,21 +2758,21 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Pack Standard (4 affiches, 12 publications, 2 vidéos, maintenance)</t>
+          <t>Gestion de la page Facebook</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Pack Standard (4 affiches, 12 publications, 2 vidéos, maintenance)</t>
+          <t>Gestion de la page Facebook · Basique</t>
         </is>
       </c>
       <c r="E59" s="8" t="n">
-        <v>50000</v>
+        <v>7000</v>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
@@ -2788,21 +2788,21 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Pack Premium (6 affiches, 20 publications, 4 vidéos, maintenance)</t>
+          <t>Gestion de la page Facebook</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Pack Premium (6 affiches, 20 publications, 4 vidéos, maintenance)</t>
+          <t>Gestion de la page Facebook · Standard</t>
         </is>
       </c>
       <c r="E60" s="8" t="n">
-        <v>115000</v>
+        <v>12500</v>
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
@@ -2818,25 +2818,25 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack</t>
+          <t>Gestion de la page Facebook</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack · Basique</t>
+          <t>Gestion de la page Facebook · Premium</t>
         </is>
       </c>
       <c r="E61" s="8" t="n">
-        <v>15000</v>
+        <v>22000</v>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
@@ -2848,25 +2848,25 @@
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack</t>
+          <t>Gestion du compte Instagram</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack · Standard</t>
+          <t>Gestion du compte Instagram · Basique</t>
         </is>
       </c>
       <c r="E62" s="8" t="n">
-        <v>28000</v>
+        <v>8000</v>
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
@@ -2878,37 +2878,67 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Site + facture avec un pack</t>
+          <t>Gestion du compte Instagram</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Gestion du compte Instagram · Standard</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>Visuo</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Gestion du compte Instagram</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>Site + facture avec un pack · Premium</t>
-        </is>
-      </c>
-      <c r="E63" s="8" t="n">
-        <v>50000</v>
-      </c>
-      <c r="F63" s="7" t="inlineStr">
-        <is>
-          <t>Unique</t>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Gestion du compte Instagram · Premium</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="n">
+        <v>24500</v>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Automatisation</t>
+          <t>Gestion du compte WhatsApp Business</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
@@ -2918,27 +2948,27 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>Automatisation · Basique</t>
+          <t>Gestion du compte WhatsApp Business · Basique</t>
         </is>
       </c>
       <c r="E65" s="8" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Automatisation</t>
+          <t>Gestion du compte WhatsApp Business</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
@@ -2948,27 +2978,27 @@
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Automatisation · Standard</t>
+          <t>Gestion du compte WhatsApp Business · Standard</t>
         </is>
       </c>
       <c r="E66" s="8" t="n">
-        <v>15000</v>
+        <v>11500</v>
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Automatisation</t>
+          <t>Gestion du compte WhatsApp Business</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
@@ -2978,193 +3008,163 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Automatisation · Premium</t>
+          <t>Gestion du compte WhatsApp Business · Premium</t>
         </is>
       </c>
       <c r="E67" s="8" t="n">
-        <v>30000</v>
+        <v>20500</v>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp</t>
+          <t>Pack Starter (Facebook ; 1 affiche, 4 publications)</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp · Basique</t>
+          <t>Pack Starter (Facebook ; 1 affiche, 4 publications)</t>
         </is>
       </c>
       <c r="E68" s="8" t="n">
-        <v>15000</v>
+        <v>6000</v>
       </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp</t>
+          <t>Pack Basique (Facebook + WhatsApp Business ; 2 affiches, 8 publications, 1 vidéo)</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp · Standard</t>
+          <t>Pack Basique (Facebook + WhatsApp Business ; 2 affiches, 8 publications, 1 vidéo)</t>
         </is>
       </c>
       <c r="E69" s="8" t="n">
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp</t>
+          <t>Pack Standard (Facebook + Instagram + WhatsApp Business ; 4 affiches, 12 publications, 2 vidéos, maintenance du site)</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Bot WhatsApp · Premium</t>
+          <t>Pack Standard (Facebook + Instagram + WhatsApp Business ; 4 affiches, 12 publications, 2 vidéos, maintenance du site)</t>
         </is>
       </c>
       <c r="E70" s="8" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Logiciel de gestion</t>
+          <t>Pack Premium (Facebook + Instagram + WhatsApp Business ; 6 affiches, 20 publications, 4 vidéos, maintenance du site)</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Basique</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Logiciel de gestion · Basique</t>
+          <t>Pack Premium (Facebook + Instagram + WhatsApp Business ; 6 affiches, 20 publications, 4 vidéos, maintenance du site)</t>
         </is>
       </c>
       <c r="E71" s="8" t="n">
-        <v>45000</v>
+        <v>115000</v>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Mensuel</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>Logia</t>
+          <t>Visuo</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Logiciel de gestion</t>
+          <t>Pack Vitrine (site vitrine Basique + 1er mois du Pack Basique, puis 18 000 / mois)</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Pack</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>Logiciel de gestion · Standard</t>
+          <t>Pack Vitrine (site vitrine Basique + 1er mois du Pack Basique, puis 18 000 / mois)</t>
         </is>
       </c>
       <c r="E72" s="8" t="n">
-        <v>90000</v>
+        <v>28000</v>
       </c>
       <c r="F72" s="7" t="inlineStr">
-        <is>
-          <t>Unique</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="7" t="inlineStr">
-        <is>
-          <t>Logia</t>
-        </is>
-      </c>
-      <c r="B73" s="7" t="inlineStr">
-        <is>
-          <t>Logiciel de gestion</t>
-        </is>
-      </c>
-      <c r="C73" s="7" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t>Logiciel de gestion · Premium</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F73" s="7" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
@@ -3178,7 +3178,7 @@
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>Suivi</t>
+          <t>Automatisation</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
@@ -3188,15 +3188,15 @@
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>Suivi · Basique</t>
+          <t>Automatisation · Basique</t>
         </is>
       </c>
       <c r="E74" s="8" t="n">
-        <v>5000</v>
+        <v>7500</v>
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Suivi</t>
+          <t>Automatisation</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
@@ -3218,15 +3218,15 @@
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>Suivi · Standard</t>
+          <t>Automatisation · Standard</t>
         </is>
       </c>
       <c r="E75" s="8" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>Suivi</t>
+          <t>Automatisation</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
@@ -3248,15 +3248,15 @@
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>Suivi · Premium</t>
+          <t>Automatisation · Premium</t>
         </is>
       </c>
       <c r="E76" s="8" t="n">
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3268,21 +3268,21 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter : mise en service</t>
+          <t>Bot WhatsApp</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter : mise en service</t>
+          <t>Bot WhatsApp · Basique</t>
         </is>
       </c>
       <c r="E77" s="8" t="n">
-        <v>7500</v>
+        <v>15000</v>
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
@@ -3298,25 +3298,25 @@
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter : suivi</t>
+          <t>Bot WhatsApp</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>Pack Starter : suivi</t>
+          <t>Bot WhatsApp · Standard</t>
         </is>
       </c>
       <c r="E78" s="8" t="n">
-        <v>5000</v>
+        <v>30000</v>
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3328,21 +3328,21 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Pack Business : mise en service</t>
+          <t>Bot WhatsApp</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>Pack Business : mise en service</t>
+          <t>Bot WhatsApp · Premium</t>
         </is>
       </c>
       <c r="E79" s="8" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
@@ -3358,25 +3358,25 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>Pack Business : suivi</t>
+          <t>Logiciel de gestion</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Basique</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>Pack Business : suivi</t>
+          <t>Logiciel de gestion · Basique</t>
         </is>
       </c>
       <c r="E80" s="8" t="n">
-        <v>10000</v>
+        <v>45000</v>
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>Mensuel</t>
+          <t>Unique</t>
         </is>
       </c>
     </row>
@@ -3388,21 +3388,21 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Pack Entreprise : mise en service</t>
+          <t>Logiciel de gestion</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Pack</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>Pack Entreprise : mise en service</t>
+          <t>Logiciel de gestion · Standard</t>
         </is>
       </c>
       <c r="E81" s="8" t="n">
-        <v>110000</v>
+        <v>90000</v>
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
@@ -3418,23 +3418,293 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
+          <t>Logiciel de gestion</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Logiciel de gestion · Premium</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="n">
+        <v>180000</v>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Suivi</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Basique</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Suivi · Basique</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Suivi</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>Suivi · Standard</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F84" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Suivi</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>Suivi · Premium</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Pack Starter : mise en service</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>Pack Starter : mise en service</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F86" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Pack Starter : suivi</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>Pack Starter : suivi</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Pack Business : mise en service</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr">
+        <is>
+          <t>Pack Business : mise en service</t>
+        </is>
+      </c>
+      <c r="E88" s="8" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F88" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Pack Business : suivi</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>Pack Business : suivi</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>Mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>Pack Entreprise : mise en service</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>Pack Entreprise : mise en service</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="n">
+        <v>110000</v>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>Logia</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
           <t>Pack Entreprise : suivi</t>
         </is>
       </c>
-      <c r="C82" s="7" t="inlineStr">
+      <c r="C91" s="7" t="inlineStr">
         <is>
           <t>Pack</t>
         </is>
       </c>
-      <c r="D82" s="7" t="inlineStr">
+      <c r="D91" s="7" t="inlineStr">
         <is>
           <t>Pack Entreprise : suivi</t>
         </is>
       </c>
-      <c r="E82" s="8" t="n">
+      <c r="E91" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="F82" s="7" t="inlineStr">
+      <c r="F91" s="7" t="inlineStr">
         <is>
           <t>Mensuel</t>
         </is>

</xml_diff>

<commit_message>
Semaine 47 (4 nouvelles mises en page) ; classeur devis/factures au nouveau logo
- Affiches : CV + lettre annotés, 3 erreurs d'exposé, grille de logos
  Visuo, parrainage en chiffre clé ; images jamais publiées.
- Classeur DWTS_Devis_Factures.xlsx régénéré : grille DWTS (version A)
  sur les devis et factures, logos transparents posés sur fond blanc.
- README : 4 mises en page ajoutées au catalogue, journal mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KbGiktRWXap9n5rdpaZ3jT
</commit_message>
<xml_diff>
--- a/outils-factures/DWTS_Devis_Factures.xlsx
+++ b/outils-factures/DWTS_Devis_Factures.xlsx
@@ -456,7 +456,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="666750" cy="533400"/>
+    <ext cx="666750" cy="666750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -511,7 +511,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="666750" cy="533400"/>
+    <ext cx="666750" cy="666750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -566,7 +566,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="523875" cy="419100"/>
+    <ext cx="523875" cy="523875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -621,7 +621,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="523875" cy="419100"/>
+    <ext cx="523875" cy="523875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -676,7 +676,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="523875" cy="419100"/>
+    <ext cx="523875" cy="523875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>

</xml_diff>

<commit_message>
Factures au seul logo du service ; vidéo de présentation v3 (nouveau logo)
- Factures (classeur Excel et PDF automatiques du script Google) : le
  logo DWTS est retiré, seul le logo de DEX, Visuo ou Logia reste. Les
  devis gardent les deux logos.
- Vidéo de présentation v3, validée par Elie : nouveau logo DWTS et bleu
  du logo à la place de l'orange ; son et minutage inchangés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KbGiktRWXap9n5rdpaZ3jT
</commit_message>
<xml_diff>
--- a/outils-factures/DWTS_Devis_Factures.xlsx
+++ b/outils-factures/DWTS_Devis_Factures.xlsx
@@ -559,31 +559,6 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>3</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="523875" cy="523875"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -614,31 +589,6 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>3</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="523875" cy="523875"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -659,31 +609,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>3</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="523875" cy="523875"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>

</xml_diff>